<commit_message>
Opties verder uitgewerkt en test cases toegeveogd
</commit_message>
<xml_diff>
--- a/GIO-Locatie_opties.xlsx
+++ b/GIO-Locatie_opties.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24729"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24827"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\DSO\Geonovum\GitHub\dso_gio_qgis_plugin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0F41519-AAE9-4E41-8090-7D83AAC2E1C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{188F1E94-5ED0-4C86-8C97-5CFF634F1B3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{326E7035-F43E-4130-9C0D-37747AF6C798}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="1" xr2:uid="{326E7035-F43E-4130-9C0D-37747AF6C798}"/>
   </bookViews>
   <sheets>
-    <sheet name="Blad1" sheetId="1" r:id="rId1"/>
+    <sheet name="Overzicht mogelijkheden" sheetId="1" r:id="rId1"/>
+    <sheet name="Test" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -103,7 +104,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="118">
   <si>
     <t>1 GIO met 1 Locatie</t>
   </si>
@@ -192,10 +193,6 @@
 (voor elke waarde 1 met features samengesmolten tot 1 Locatie)</t>
   </si>
   <si>
-    <t>1 GIO met meerdere locaties
-(voor elke waarde een Locatie)</t>
-  </si>
-  <si>
     <t>1 GIO met 1 locatie
 (features met gekozen waarde in attribuut samengesmolten tot 1 locatie)</t>
   </si>
@@ -205,13 +202,419 @@
   </si>
   <si>
     <t>attribuutwaardelijst&lt;&gt;''</t>
+  </si>
+  <si>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>Inputbestand bevat meerdere features met in elk geval 1 attribuut met unieke en 1 attribuut met meerdere dubbele waarden</t>
+  </si>
+  <si>
+    <t>Bouwhoogte GIO van gemeentestad:</t>
+  </si>
+  <si>
+    <t>4 features</t>
+  </si>
+  <si>
+    <t>attribuut Naam met unieke namen voor elk feature</t>
+  </si>
+  <si>
+    <t>attribuut kwantitatieveNormwaarde met 2 waarden</t>
+  </si>
+  <si>
+    <t>Naam</t>
+  </si>
+  <si>
+    <t>kwantitatieveNormwaarde</t>
+  </si>
+  <si>
+    <t>Zuilichem industriegebied 1</t>
+  </si>
+  <si>
+    <t>Zuilichem industriegebied 2</t>
+  </si>
+  <si>
+    <t>Zuilichem industriegebied 3</t>
+  </si>
+  <si>
+    <t>Zuilichem industriegebied 4</t>
+  </si>
+  <si>
+    <t>B5</t>
+  </si>
+  <si>
+    <t>FRBRExpression</t>
+  </si>
+  <si>
+    <t>Locatie</t>
+  </si>
+  <si>
+    <t>GML</t>
+  </si>
+  <si>
+    <t>Filter?</t>
+  </si>
+  <si>
+    <t>Attribuut</t>
+  </si>
+  <si>
+    <t>LosseGIOs?</t>
+  </si>
+  <si>
+    <t>Waarde</t>
+  </si>
+  <si>
+    <t>/join/id/regdata/gm0297/2022/test/nld@2022;1</t>
+  </si>
+  <si>
+    <t>Bouwhoogte</t>
+  </si>
+  <si>
+    <t>Nee</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Ja</t>
+  </si>
+  <si>
+    <t>1 GIO met meerdere locaties
+(voor elke waarde 1 met features samengesmolten tot 1 Locatie)</t>
+  </si>
+  <si>
+    <t>Cel</t>
+  </si>
+  <si>
+    <t>Selectie?</t>
+  </si>
+  <si>
+    <t>C3</t>
+  </si>
+  <si>
+    <t>Gelijk aan B3 omdat eerst wordt samengesmolten</t>
+  </si>
+  <si>
+    <t>Aantal GIO's</t>
+  </si>
+  <si>
+    <t>Naam GIO's</t>
+  </si>
+  <si>
+    <t>Waarde van Naam</t>
+  </si>
+  <si>
+    <t>Aantal locaties</t>
+  </si>
+  <si>
+    <t>Naam locaties</t>
+  </si>
+  <si>
+    <t>Opmerking</t>
+  </si>
+  <si>
+    <t>alle vlakken zijn samengesmolten</t>
+  </si>
+  <si>
+    <t>alleen geselecteerde vlakken (samengesmolten)</t>
+  </si>
+  <si>
+    <t>7 en 13</t>
+  </si>
+  <si>
+    <t>C5</t>
+  </si>
+  <si>
+    <t>Waarde van kwantitatieveNormwaarde</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>D3</t>
+  </si>
+  <si>
+    <t>Bouwhoogte + volgnummer</t>
+  </si>
+  <si>
+    <t>b.v. Bouwhoogte_1</t>
+  </si>
+  <si>
+    <t>D5</t>
+  </si>
+  <si>
+    <t>E3</t>
+  </si>
+  <si>
+    <t>E4</t>
+  </si>
+  <si>
+    <t>E5</t>
+  </si>
+  <si>
+    <t>7.gml</t>
+  </si>
+  <si>
+    <t>7 (2x) en 13 (2x)</t>
+  </si>
+  <si>
+    <t>kwantitatieve-
+Normwaarde</t>
+  </si>
+  <si>
+    <t>Features 
+samensmelten</t>
+  </si>
+  <si>
+    <t>FRBRExpression
+6e deel</t>
+  </si>
+  <si>
+    <t>test</t>
+  </si>
+  <si>
+    <t>test_&lt;volgnummer&gt;</t>
+  </si>
+  <si>
+    <r>
+      <t>/join/id/regdata/gm0297/2022/</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;Naam&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>/nld@2022;1</t>
+    </r>
+  </si>
+  <si>
+    <t>7.gml en 13.gml</t>
+  </si>
+  <si>
+    <t>b.v. Zuilichem industriegebied 1</t>
+  </si>
+  <si>
+    <t>&lt;Naam&gt;</t>
+  </si>
+  <si>
+    <t>Kies laag: Bouwhoogte_—_gio</t>
+  </si>
+  <si>
+    <t>Kies gml bestand: Bouwhoogte_&lt;testnr&gt;.gml</t>
+  </si>
+  <si>
+    <t>B3a</t>
+  </si>
+  <si>
+    <t>B3b</t>
+  </si>
+  <si>
+    <t>B4a</t>
+  </si>
+  <si>
+    <t>B4b</t>
+  </si>
+  <si>
+    <t>C4a</t>
+  </si>
+  <si>
+    <t>C4b</t>
+  </si>
+  <si>
+    <t>D4a</t>
+  </si>
+  <si>
+    <t>D4b</t>
+  </si>
+  <si>
+    <t>Bouwhoogte_B3a.gml</t>
+  </si>
+  <si>
+    <t>Bouwhoogte_B3b.gml</t>
+  </si>
+  <si>
+    <t>Bouwhoogte_B4a.gml</t>
+  </si>
+  <si>
+    <t>Bouwhoogte_B4b.gml</t>
+  </si>
+  <si>
+    <t>Bouwhoogte_B5.gml</t>
+  </si>
+  <si>
+    <t>Bouwhoogte_C3.gml</t>
+  </si>
+  <si>
+    <t>Bouwhoogte_D3.gml</t>
+  </si>
+  <si>
+    <t>Bouwhoogte_D4a.gml</t>
+  </si>
+  <si>
+    <t>Bouwhoogte_D4b.gml</t>
+  </si>
+  <si>
+    <t>Bouwhoogte_D5.gml</t>
+  </si>
+  <si>
+    <r>
+      <t>Bouwhoogte_E3_</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;volgnummer&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.gml</t>
+    </r>
+  </si>
+  <si>
+    <t>Bouwhoogte_C5.gml</t>
+  </si>
+  <si>
+    <r>
+      <t>Bouwhoogte_C4a_</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;Naam&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.gml</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Bouwhoogte_C4b_</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;Naam&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.gml</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Bouwhoogte_E4_</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;kwantitatieveNormwaarde&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.gml</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Bouwhoogte_E5_</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;kwantitatieveNormwaarde&gt;_&lt;volgnummer&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.gml</t>
+    </r>
+  </si>
+  <si>
+    <t>b.v. Bouwhoogte_E3_1.gml</t>
+  </si>
+  <si>
+    <t>kwantitatievenormwaarde_7_1.gml</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="13" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -307,6 +710,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="11">
     <fill>
@@ -370,7 +781,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -514,11 +925,55 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -556,12 +1011,6 @@
     <xf numFmtId="0" fontId="7" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -599,6 +1048,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -613,12 +1068,49 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
@@ -1000,31 +1492,27 @@
   <sheetData>
     <row r="1" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="28"/>
-      <c r="B1" s="13" t="s">
+      <c r="B1" s="32" t="s">
         <v>7</v>
       </c>
-      <c r="C1" s="13" t="s">
-        <v>7</v>
-      </c>
-      <c r="D1" s="14" t="s">
+      <c r="C1" s="33"/>
+      <c r="D1" s="34" t="s">
         <v>8</v>
       </c>
-      <c r="E1" s="14" t="s">
-        <v>8</v>
-      </c>
+      <c r="E1" s="35"/>
     </row>
     <row r="2" spans="1:6" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="29"/>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="16" t="s">
+      <c r="C2" s="14" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="16" t="s">
+      <c r="E2" s="14" t="s">
         <v>10</v>
       </c>
     </row>
@@ -1046,11 +1534,11 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="15" t="s">
         <v>5</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>26</v>
@@ -1058,7 +1546,7 @@
       <c r="D4" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E4" s="32" t="s">
+      <c r="E4" s="26" t="s">
         <v>23</v>
       </c>
     </row>
@@ -1070,10 +1558,10 @@
         <v>1</v>
       </c>
       <c r="C5" s="3" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="4" t="s">
         <v>28</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>29</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>3</v>
@@ -1084,72 +1572,72 @@
       <c r="A7" s="30" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="23" t="s">
+      <c r="C7" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="18" t="s">
+      <c r="D7" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="19" t="s">
+      <c r="E7" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="19" t="s">
+      <c r="F7" s="17" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="31"/>
-      <c r="B8" s="25" t="s">
+      <c r="B8" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="24" t="s">
+      <c r="C8" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="D8" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="E8" s="20" t="s">
+      <c r="E8" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="20"/>
+      <c r="F8" s="18"/>
     </row>
     <row r="9" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="31"/>
-      <c r="B9" s="25" t="s">
+      <c r="B9" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="C9" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="18" t="s">
+      <c r="D9" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="19" t="s">
+      <c r="E9" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="F9" s="19" t="s">
+      <c r="F9" s="17" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="31"/>
-      <c r="B10" s="33" t="s">
+      <c r="B10" s="27" t="s">
         <v>21</v>
       </c>
-      <c r="C10" s="24" t="s">
+      <c r="C10" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="18" t="s">
+      <c r="D10" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="21" t="s">
+      <c r="E10" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="21" t="s">
-        <v>30</v>
+      <c r="F10" s="19" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1157,147 +1645,149 @@
       <c r="A12" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="B12" s="26" t="s">
+      <c r="B12" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="23" t="s">
+      <c r="C12" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="D12" s="22" t="s">
+      <c r="D12" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="E12" s="20" t="s">
+      <c r="E12" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="F12" s="20"/>
+      <c r="F12" s="18"/>
     </row>
     <row r="13" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="31"/>
-      <c r="B13" s="26" t="s">
+      <c r="B13" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="C13" s="23" t="s">
+      <c r="C13" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="D13" s="22" t="s">
+      <c r="D13" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="E13" s="21" t="s">
+      <c r="E13" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="F13" s="21" t="s">
-        <v>30</v>
+      <c r="F13" s="19" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="31"/>
-      <c r="B14" s="26" t="s">
+      <c r="B14" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="C14" s="23" t="s">
+      <c r="C14" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="D14" s="18" t="s">
+      <c r="D14" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="E14" s="20" t="s">
+      <c r="E14" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="F14" s="20"/>
+      <c r="F14" s="18"/>
     </row>
     <row r="15" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="31"/>
-      <c r="B15" s="26" t="s">
+      <c r="B15" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="C15" s="23" t="s">
+      <c r="C15" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="D15" s="18" t="s">
+      <c r="D15" s="16" t="s">
         <v>16</v>
       </c>
-      <c r="E15" s="21" t="s">
+      <c r="E15" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="F15" s="21" t="s">
-        <v>30</v>
+      <c r="F15" s="19" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="16" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="31"/>
-      <c r="B16" s="27" t="s">
+      <c r="B16" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="23" t="s">
+      <c r="C16" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="D16" s="22" t="s">
+      <c r="D16" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="E16" s="19" t="s">
+      <c r="E16" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="F16" s="19" t="s">
+      <c r="F16" s="17" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="31"/>
-      <c r="B17" s="27" t="s">
+      <c r="B17" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="C17" s="24" t="s">
+      <c r="C17" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="D17" s="22" t="s">
+      <c r="D17" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="E17" s="20" t="s">
+      <c r="E17" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="F17" s="20"/>
+      <c r="F17" s="18"/>
     </row>
     <row r="18" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="31"/>
-      <c r="B18" s="27" t="s">
+      <c r="B18" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="24" t="s">
+      <c r="C18" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="D18" s="22" t="s">
+      <c r="D18" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="E18" s="19" t="s">
+      <c r="E18" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="F18" s="19" t="s">
+      <c r="F18" s="17" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="31"/>
-      <c r="B19" s="27" t="s">
+      <c r="B19" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="C19" s="24" t="s">
+      <c r="C19" s="22" t="s">
         <v>15</v>
       </c>
-      <c r="D19" s="22" t="s">
+      <c r="D19" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="E19" s="21" t="s">
+      <c r="E19" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="F19" s="21" t="s">
-        <v>30</v>
+      <c r="F19" s="19" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="5">
     <mergeCell ref="A1:A2"/>
     <mergeCell ref="A7:A10"/>
     <mergeCell ref="A12:A19"/>
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="D1:E1"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1305,4 +1795,949 @@
   <drawing r:id="rId2"/>
   <legacyDrawing r:id="rId3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AA4DA3F-D43D-4869-BF17-622F549546C1}">
+  <dimension ref="A1:O32"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="48.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="4.7109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="3.7109375" style="39" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="62" style="41" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="22.85546875" style="41" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="3.7109375" style="41" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="36.5703125" style="41" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="46" style="44" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="46" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="11" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="22.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B1" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="C1" s="37"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B2" s="37" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="37"/>
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B3" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="37"/>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B4" s="37" t="s">
+        <v>34</v>
+      </c>
+      <c r="C4" s="37"/>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B5" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="37"/>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B6" s="46"/>
+      <c r="C6" s="46"/>
+    </row>
+    <row r="7" spans="1:15" s="47" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B7" s="47" t="s">
+        <v>90</v>
+      </c>
+      <c r="J7" s="49"/>
+      <c r="O7" s="50"/>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B8" s="48" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" s="38" customFormat="1" ht="74.25" x14ac:dyDescent="0.25">
+      <c r="B9" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="C9" s="51" t="s">
+        <v>81</v>
+      </c>
+      <c r="J9" s="40"/>
+      <c r="K9" s="42"/>
+      <c r="L9" s="42"/>
+      <c r="M9" s="42"/>
+      <c r="N9" s="42"/>
+      <c r="O9" s="45"/>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B10" s="36" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="36">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B11" s="36" t="s">
+        <v>39</v>
+      </c>
+      <c r="C11" s="36">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B12" s="36" t="s">
+        <v>40</v>
+      </c>
+      <c r="C12" s="36">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B13" s="36" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" s="36">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>56</v>
+      </c>
+      <c r="B15" t="s">
+        <v>45</v>
+      </c>
+      <c r="D15" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16" spans="1:15" s="38" customFormat="1" ht="79.5" x14ac:dyDescent="0.25">
+      <c r="B16" s="38" t="s">
+        <v>43</v>
+      </c>
+      <c r="C16" s="38" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" s="38" t="s">
+        <v>46</v>
+      </c>
+      <c r="E16" s="38" t="s">
+        <v>47</v>
+      </c>
+      <c r="F16" s="38" t="s">
+        <v>49</v>
+      </c>
+      <c r="G16" s="38" t="s">
+        <v>48</v>
+      </c>
+      <c r="H16" s="51" t="s">
+        <v>82</v>
+      </c>
+      <c r="I16" s="38" t="s">
+        <v>57</v>
+      </c>
+      <c r="J16" s="40" t="s">
+        <v>60</v>
+      </c>
+      <c r="K16" s="42" t="s">
+        <v>61</v>
+      </c>
+      <c r="L16" s="51" t="s">
+        <v>83</v>
+      </c>
+      <c r="M16" s="42" t="s">
+        <v>63</v>
+      </c>
+      <c r="N16" s="42" t="s">
+        <v>64</v>
+      </c>
+      <c r="O16" s="45" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>92</v>
+      </c>
+      <c r="B17" t="s">
+        <v>50</v>
+      </c>
+      <c r="C17" t="s">
+        <v>51</v>
+      </c>
+      <c r="D17" t="s">
+        <v>52</v>
+      </c>
+      <c r="E17" t="s">
+        <v>53</v>
+      </c>
+      <c r="F17" t="s">
+        <v>53</v>
+      </c>
+      <c r="G17" t="s">
+        <v>52</v>
+      </c>
+      <c r="H17" t="s">
+        <v>54</v>
+      </c>
+      <c r="I17" t="s">
+        <v>52</v>
+      </c>
+      <c r="J17" s="39">
+        <v>1</v>
+      </c>
+      <c r="K17" s="41" t="s">
+        <v>100</v>
+      </c>
+      <c r="L17" t="s">
+        <v>84</v>
+      </c>
+      <c r="M17" s="41">
+        <v>1</v>
+      </c>
+      <c r="N17" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="O17" s="44" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="18" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>93</v>
+      </c>
+      <c r="B18" t="s">
+        <v>50</v>
+      </c>
+      <c r="C18" t="s">
+        <v>51</v>
+      </c>
+      <c r="D18" t="s">
+        <v>52</v>
+      </c>
+      <c r="E18" t="s">
+        <v>53</v>
+      </c>
+      <c r="F18" t="s">
+        <v>53</v>
+      </c>
+      <c r="G18" t="s">
+        <v>52</v>
+      </c>
+      <c r="H18" t="s">
+        <v>54</v>
+      </c>
+      <c r="I18" t="s">
+        <v>54</v>
+      </c>
+      <c r="J18" s="39">
+        <v>1</v>
+      </c>
+      <c r="K18" s="41" t="s">
+        <v>101</v>
+      </c>
+      <c r="L18" t="s">
+        <v>84</v>
+      </c>
+      <c r="M18" s="41">
+        <v>1</v>
+      </c>
+      <c r="N18" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="O18" s="44" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="19" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>94</v>
+      </c>
+      <c r="B19" t="s">
+        <v>50</v>
+      </c>
+      <c r="C19" t="s">
+        <v>51</v>
+      </c>
+      <c r="D19" t="s">
+        <v>54</v>
+      </c>
+      <c r="E19" t="s">
+        <v>36</v>
+      </c>
+      <c r="F19" t="s">
+        <v>53</v>
+      </c>
+      <c r="G19" t="s">
+        <v>52</v>
+      </c>
+      <c r="H19" t="s">
+        <v>54</v>
+      </c>
+      <c r="I19" t="s">
+        <v>52</v>
+      </c>
+      <c r="J19" s="39">
+        <v>1</v>
+      </c>
+      <c r="K19" s="41" t="s">
+        <v>102</v>
+      </c>
+      <c r="L19" t="s">
+        <v>84</v>
+      </c>
+      <c r="M19" s="41">
+        <v>4</v>
+      </c>
+      <c r="N19" s="43" t="s">
+        <v>62</v>
+      </c>
+      <c r="O19" s="44" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="20" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>95</v>
+      </c>
+      <c r="B20" t="s">
+        <v>50</v>
+      </c>
+      <c r="C20" t="s">
+        <v>51</v>
+      </c>
+      <c r="D20" t="s">
+        <v>54</v>
+      </c>
+      <c r="E20" t="s">
+        <v>37</v>
+      </c>
+      <c r="F20" t="s">
+        <v>53</v>
+      </c>
+      <c r="G20" t="s">
+        <v>52</v>
+      </c>
+      <c r="H20" t="s">
+        <v>54</v>
+      </c>
+      <c r="I20" t="s">
+        <v>52</v>
+      </c>
+      <c r="J20" s="39">
+        <v>1</v>
+      </c>
+      <c r="K20" s="41" t="s">
+        <v>103</v>
+      </c>
+      <c r="L20" t="s">
+        <v>84</v>
+      </c>
+      <c r="M20" s="43">
+        <v>2</v>
+      </c>
+      <c r="N20" s="43" t="s">
+        <v>70</v>
+      </c>
+      <c r="O20" s="44" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="21" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>42</v>
+      </c>
+      <c r="B21" t="s">
+        <v>50</v>
+      </c>
+      <c r="C21" t="s">
+        <v>51</v>
+      </c>
+      <c r="D21" t="s">
+        <v>54</v>
+      </c>
+      <c r="E21" t="s">
+        <v>37</v>
+      </c>
+      <c r="F21">
+        <v>7</v>
+      </c>
+      <c r="G21" t="s">
+        <v>52</v>
+      </c>
+      <c r="H21" t="s">
+        <v>54</v>
+      </c>
+      <c r="I21" t="s">
+        <v>52</v>
+      </c>
+      <c r="J21" s="39">
+        <v>1</v>
+      </c>
+      <c r="K21" s="41" t="s">
+        <v>104</v>
+      </c>
+      <c r="L21" t="s">
+        <v>84</v>
+      </c>
+      <c r="M21" s="43">
+        <v>1</v>
+      </c>
+      <c r="N21" s="43" t="s">
+        <v>70</v>
+      </c>
+      <c r="O21" s="44">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>58</v>
+      </c>
+      <c r="B22" t="s">
+        <v>50</v>
+      </c>
+      <c r="C22" t="s">
+        <v>51</v>
+      </c>
+      <c r="D22" t="s">
+        <v>52</v>
+      </c>
+      <c r="E22" t="s">
+        <v>53</v>
+      </c>
+      <c r="F22" t="s">
+        <v>53</v>
+      </c>
+      <c r="G22" t="s">
+        <v>54</v>
+      </c>
+      <c r="H22" t="s">
+        <v>54</v>
+      </c>
+      <c r="I22" t="s">
+        <v>52</v>
+      </c>
+      <c r="J22" s="39">
+        <v>1</v>
+      </c>
+      <c r="K22" s="41" t="s">
+        <v>105</v>
+      </c>
+      <c r="L22" t="s">
+        <v>84</v>
+      </c>
+      <c r="M22" s="43">
+        <v>1</v>
+      </c>
+      <c r="N22" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="O22" s="44" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="23" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>96</v>
+      </c>
+      <c r="B23" t="s">
+        <v>50</v>
+      </c>
+      <c r="C23" t="s">
+        <v>51</v>
+      </c>
+      <c r="D23" t="s">
+        <v>54</v>
+      </c>
+      <c r="E23" t="s">
+        <v>36</v>
+      </c>
+      <c r="F23" t="s">
+        <v>53</v>
+      </c>
+      <c r="G23" t="s">
+        <v>54</v>
+      </c>
+      <c r="H23" t="s">
+        <v>54</v>
+      </c>
+      <c r="I23" t="s">
+        <v>52</v>
+      </c>
+      <c r="J23" s="39">
+        <v>4</v>
+      </c>
+      <c r="K23" s="43" t="s">
+        <v>112</v>
+      </c>
+      <c r="L23" t="s">
+        <v>85</v>
+      </c>
+      <c r="M23" s="43">
+        <v>1</v>
+      </c>
+      <c r="N23" s="43" t="s">
+        <v>62</v>
+      </c>
+      <c r="O23" s="44" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="24" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>97</v>
+      </c>
+      <c r="B24" t="s">
+        <v>86</v>
+      </c>
+      <c r="C24" t="s">
+        <v>51</v>
+      </c>
+      <c r="D24" t="s">
+        <v>54</v>
+      </c>
+      <c r="E24" t="s">
+        <v>36</v>
+      </c>
+      <c r="F24" t="s">
+        <v>53</v>
+      </c>
+      <c r="G24" t="s">
+        <v>54</v>
+      </c>
+      <c r="H24" t="s">
+        <v>54</v>
+      </c>
+      <c r="I24" t="s">
+        <v>52</v>
+      </c>
+      <c r="J24" s="39">
+        <v>4</v>
+      </c>
+      <c r="K24" s="43" t="s">
+        <v>113</v>
+      </c>
+      <c r="L24" t="s">
+        <v>89</v>
+      </c>
+      <c r="M24" s="43">
+        <v>1</v>
+      </c>
+      <c r="N24" s="43" t="s">
+        <v>62</v>
+      </c>
+      <c r="O24" s="44" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="25" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>69</v>
+      </c>
+      <c r="B25" t="s">
+        <v>50</v>
+      </c>
+      <c r="C25" t="s">
+        <v>51</v>
+      </c>
+      <c r="D25" t="s">
+        <v>54</v>
+      </c>
+      <c r="E25" t="s">
+        <v>37</v>
+      </c>
+      <c r="F25">
+        <v>7</v>
+      </c>
+      <c r="G25" t="s">
+        <v>54</v>
+      </c>
+      <c r="H25" t="s">
+        <v>54</v>
+      </c>
+      <c r="I25" t="s">
+        <v>52</v>
+      </c>
+      <c r="J25" s="39">
+        <v>1</v>
+      </c>
+      <c r="K25" s="52" t="s">
+        <v>111</v>
+      </c>
+      <c r="L25" t="s">
+        <v>84</v>
+      </c>
+      <c r="M25" s="43">
+        <v>1</v>
+      </c>
+      <c r="N25" s="43" t="s">
+        <v>70</v>
+      </c>
+      <c r="O25" s="44" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="26" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>72</v>
+      </c>
+      <c r="B26" t="s">
+        <v>50</v>
+      </c>
+      <c r="C26" t="s">
+        <v>51</v>
+      </c>
+      <c r="D26" t="s">
+        <v>52</v>
+      </c>
+      <c r="E26" t="s">
+        <v>53</v>
+      </c>
+      <c r="F26" t="s">
+        <v>53</v>
+      </c>
+      <c r="G26" t="s">
+        <v>52</v>
+      </c>
+      <c r="H26" t="s">
+        <v>52</v>
+      </c>
+      <c r="I26" t="s">
+        <v>52</v>
+      </c>
+      <c r="J26" s="39">
+        <v>1</v>
+      </c>
+      <c r="K26" s="41" t="s">
+        <v>106</v>
+      </c>
+      <c r="L26" t="s">
+        <v>84</v>
+      </c>
+      <c r="M26" s="43">
+        <v>4</v>
+      </c>
+      <c r="N26" s="43" t="s">
+        <v>73</v>
+      </c>
+      <c r="O26" s="44" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="27" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>98</v>
+      </c>
+      <c r="B27" t="s">
+        <v>50</v>
+      </c>
+      <c r="C27" t="s">
+        <v>51</v>
+      </c>
+      <c r="D27" t="s">
+        <v>54</v>
+      </c>
+      <c r="E27" t="s">
+        <v>36</v>
+      </c>
+      <c r="F27" t="s">
+        <v>53</v>
+      </c>
+      <c r="G27" t="s">
+        <v>52</v>
+      </c>
+      <c r="H27" t="s">
+        <v>52</v>
+      </c>
+      <c r="I27" t="s">
+        <v>52</v>
+      </c>
+      <c r="J27" s="39">
+        <v>1</v>
+      </c>
+      <c r="K27" s="41" t="s">
+        <v>107</v>
+      </c>
+      <c r="L27" t="s">
+        <v>84</v>
+      </c>
+      <c r="M27" s="43">
+        <v>4</v>
+      </c>
+      <c r="N27" s="43" t="s">
+        <v>62</v>
+      </c>
+      <c r="O27" s="44" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="28" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>99</v>
+      </c>
+      <c r="B28" t="s">
+        <v>50</v>
+      </c>
+      <c r="C28" t="s">
+        <v>51</v>
+      </c>
+      <c r="D28" t="s">
+        <v>54</v>
+      </c>
+      <c r="E28" t="s">
+        <v>37</v>
+      </c>
+      <c r="F28" t="s">
+        <v>53</v>
+      </c>
+      <c r="G28" t="s">
+        <v>52</v>
+      </c>
+      <c r="H28" t="s">
+        <v>52</v>
+      </c>
+      <c r="I28" t="s">
+        <v>52</v>
+      </c>
+      <c r="J28" s="39">
+        <v>1</v>
+      </c>
+      <c r="K28" s="41" t="s">
+        <v>108</v>
+      </c>
+      <c r="L28" t="s">
+        <v>84</v>
+      </c>
+      <c r="M28" s="43">
+        <v>4</v>
+      </c>
+      <c r="N28" s="43" t="s">
+        <v>70</v>
+      </c>
+      <c r="O28" s="44" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="29" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>75</v>
+      </c>
+      <c r="B29" t="s">
+        <v>50</v>
+      </c>
+      <c r="C29" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29" t="s">
+        <v>54</v>
+      </c>
+      <c r="E29" t="s">
+        <v>37</v>
+      </c>
+      <c r="F29">
+        <v>7</v>
+      </c>
+      <c r="G29" t="s">
+        <v>52</v>
+      </c>
+      <c r="H29" t="s">
+        <v>52</v>
+      </c>
+      <c r="I29" t="s">
+        <v>52</v>
+      </c>
+      <c r="J29" s="39">
+        <v>1</v>
+      </c>
+      <c r="K29" s="41" t="s">
+        <v>109</v>
+      </c>
+      <c r="L29" t="s">
+        <v>84</v>
+      </c>
+      <c r="M29" s="43">
+        <v>2</v>
+      </c>
+      <c r="N29" s="43" t="s">
+        <v>70</v>
+      </c>
+      <c r="O29" s="44" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="30" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>76</v>
+      </c>
+      <c r="B30" t="s">
+        <v>50</v>
+      </c>
+      <c r="C30" t="s">
+        <v>51</v>
+      </c>
+      <c r="D30" t="s">
+        <v>52</v>
+      </c>
+      <c r="E30" t="s">
+        <v>53</v>
+      </c>
+      <c r="F30" t="s">
+        <v>53</v>
+      </c>
+      <c r="G30" t="s">
+        <v>54</v>
+      </c>
+      <c r="H30" t="s">
+        <v>52</v>
+      </c>
+      <c r="I30" t="s">
+        <v>52</v>
+      </c>
+      <c r="J30" s="39">
+        <v>4</v>
+      </c>
+      <c r="K30" s="41" t="s">
+        <v>110</v>
+      </c>
+      <c r="L30" t="s">
+        <v>85</v>
+      </c>
+      <c r="M30" s="43">
+        <v>1</v>
+      </c>
+      <c r="N30" s="43" t="s">
+        <v>51</v>
+      </c>
+      <c r="O30" s="41" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="31" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>77</v>
+      </c>
+      <c r="B31" t="s">
+        <v>50</v>
+      </c>
+      <c r="C31" t="s">
+        <v>51</v>
+      </c>
+      <c r="D31" t="s">
+        <v>54</v>
+      </c>
+      <c r="E31" t="s">
+        <v>37</v>
+      </c>
+      <c r="F31" t="s">
+        <v>53</v>
+      </c>
+      <c r="G31" t="s">
+        <v>54</v>
+      </c>
+      <c r="H31" t="s">
+        <v>52</v>
+      </c>
+      <c r="I31" t="s">
+        <v>52</v>
+      </c>
+      <c r="J31" s="39">
+        <v>2</v>
+      </c>
+      <c r="K31" s="43" t="s">
+        <v>114</v>
+      </c>
+      <c r="L31" t="s">
+        <v>85</v>
+      </c>
+      <c r="M31" s="43">
+        <v>2</v>
+      </c>
+      <c r="N31" s="43" t="s">
+        <v>70</v>
+      </c>
+      <c r="O31" s="44" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="32" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>78</v>
+      </c>
+      <c r="B32" t="s">
+        <v>50</v>
+      </c>
+      <c r="C32" t="s">
+        <v>51</v>
+      </c>
+      <c r="D32" t="s">
+        <v>54</v>
+      </c>
+      <c r="E32" t="s">
+        <v>37</v>
+      </c>
+      <c r="F32">
+        <v>7</v>
+      </c>
+      <c r="G32" t="s">
+        <v>54</v>
+      </c>
+      <c r="H32" t="s">
+        <v>52</v>
+      </c>
+      <c r="I32" t="s">
+        <v>52</v>
+      </c>
+      <c r="J32" s="39">
+        <v>2</v>
+      </c>
+      <c r="K32" s="43" t="s">
+        <v>115</v>
+      </c>
+      <c r="L32" t="s">
+        <v>85</v>
+      </c>
+      <c r="M32" s="43">
+        <v>1</v>
+      </c>
+      <c r="N32" s="43" t="s">
+        <v>70</v>
+      </c>
+      <c r="O32" s="44" t="s">
+        <v>117</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B1:C1"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <ignoredErrors>
+    <ignoredError sqref="O29" numberStoredAsText="1"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>